<commit_message>
fix(docs): update default Excel knowledge base to 3 columns (Nr pytania, Pytanie, Odpowiedź)
</commit_message>
<xml_diff>
--- a/documents/knowledge_base.xlsx
+++ b/documents/knowledge_base.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="KnowledgeBase" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="FAQ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,168 +413,113 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Nr pytania</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Pytanie</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Question</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Keywords</t>
+          <t>Odpowiedź</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>KB001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Return Policy</t>
+          <t>Jaki jest czas realizacji zamówienia w sklepie?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>What is the return policy for damaged or defective items?</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Customers can return defective items within 30 days of purchase for a full refund or replacement. Return shipping is completely free for defective goods.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>refund, defective, damaged, replacement, 30 days</t>
+          <t>Standardowy czas realizacji zamówienia wynosi od 1 do 3 dni roboczych. W przypadku przesyłek ekspresowych doręczenie następuje w ciągu 24 godzin od momentu nadania.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>KB002</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Shipping</t>
+          <t>Jakie są warunki i procedury zwrotu towaru?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>How long does international shipping take and what is the cost?</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Standard international shipping takes 5-10 business days and costs . Express shipping takes 2-4 business days for .</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>international, delivery, delivery time, shipping cost, express</t>
+          <t>Klient ma prawo odstąpić od umowy i zwrócić towar w ciągu 14 dni od momentu odebrania paczki bez podawania przyczyny. Towar musi być w stanie nienaruszonym wraz z oryginalnym opakowaniem i dowodem zakupu.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>KB003</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Account &amp; Security</t>
+          <t>Jak skontaktować się z działem pomocy technicznej i obsługi klienta?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>How do I reset my password if I cannot access my two-factor authentication (2FA)?</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>If you lose access to your 2FA device, click 'Recover Account' on the login page and use your 16-character backup recovery code. Alternatively, contact support@example.com with identity verification.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2fa, two-factor, password reset, security, account recovery</t>
+          <t>Dział obsługi klienta jest dostępny od poniedziałku do piątku w godzinach 8:00 - 18:00 pod numerem telefonu +48 22 123 45 67 oraz adresem e-mail: pomoc@twojafirma.pl.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>KB004</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HR &amp; Benefits</t>
+          <t>Jakie formy płatności są akceptowane w sklepie?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>What is the annual remote work equipment stipend for employees?</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Full-time employees receive an annual remote work equipment stipend of ,000 USD, renewable every January 1st upon submitting itemized receipts.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>remote work, stipend, equipment, budget, allowance</t>
+          <t>Obsługujemy szybkie płatności BLIK, karty płatnicze Visa i Mastercard, przelewy online PayU/Przelewy24 oraz płatność przy odbiorze (za pobraniem).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>KB005</t>
-        </is>
+      <c r="A6" t="n">
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>API &amp; Integration</t>
+          <t>W jaki sposób mogę zgłosić reklamację uszkodzonego produktu?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>What are the rate limits for the public REST API endpoints?</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Free tier accounts are limited to 60 requests per minute and 5,000 requests per day. Enterprise tier accounts have custom limits up to 10,000 requests per minute.</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>api rate limit, rate limit, quota, enterprise, requests per minute</t>
+          <t>Reklamację można zgłosić drogą elektroniczną, wysyłając formularz reklamacyjny ze zdjęciem wady na adres reklamacje@twojafirma.pl. Rozpatrzenie reklamacji trwa do 14 dni roboczych.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Czy oferujecie darmową dostawę i od jakiej kwoty?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Darmowa dostawa przysługuje dla wszystkich zamówień krajowych o wartości powyżej 150 zł brutto. Dla zamówień poniżej tej kwoty koszt wysyłki kurierem wynosi 14 zł.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(security): add rate limiting, payload limits, LLM timeouts, and prompt injection defense
- Add SlowAPI IP-based rate limiting on /ask, /ask/stream, and /ingest endpoints
- Implement request body size middleware (1MB limit) and Pydantic max_length validation
- Add configurable LLM timeout and request timeout handling with HTTP 504 Gateway Timeout
- Introduce prompt injection input sanitization and delimiter tags (<context>, <user_question>)
- Harden RAG system prompt against instructions override and system prompt leakage
- Add pytest test suite for security utilities, payload limits, timeouts, and validation
</commit_message>
<xml_diff>
--- a/documents/knowledge_base.xlsx
+++ b/documents/knowledge_base.xlsx
@@ -1,34 +1,96 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kamil/Desktop/Kodowanie/RAG/documents/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B2BD4D-43D7-904E-AA0A-75B3423F7507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="19480" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="FAQ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="FAQ" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>Question No.</t>
+  </si>
+  <si>
+    <t>Question</t>
+  </si>
+  <si>
+    <t>Answer</t>
+  </si>
+  <si>
+    <t>What is the order processing time in the store?</t>
+  </si>
+  <si>
+    <t>The standard order processing time is 1 to 3 business days. For express shipments, delivery takes place within 24 hours from the moment the package is dispatched.</t>
+  </si>
+  <si>
+    <t>What are the terms and procedures for returning goods?</t>
+  </si>
+  <si>
+    <t>Customers have the right to withdraw from the contract and return goods within 14 days from the date of receiving the package without providing a reason. The product must be in an undamaged condition, with the original packaging and proof of purchase.</t>
+  </si>
+  <si>
+    <t>How can I contact technical support and customer service?</t>
+  </si>
+  <si>
+    <t>The customer service department is available Monday to Friday from 8:00 AM to 6:00 PM at phone number +48 22 123 45 67 and via email: pomoc@twojafirma.pl.</t>
+  </si>
+  <si>
+    <t>What payment methods are accepted in the store?</t>
+  </si>
+  <si>
+    <t>We support BLIK instant payments, Visa and Mastercard payment cards, online transfers via PayU/Przelewy24, and cash on delivery.</t>
+  </si>
+  <si>
+    <t>How can I submit a complaint about a damaged product?</t>
+  </si>
+  <si>
+    <t>A complaint can be submitted electronically by sending a complaint form with a photo of the defect to reklamacje@twojafirma.pl. Complaints are processed within up to 14 business days.</t>
+  </si>
+  <si>
+    <t>Do you offer free delivery and from what amount?</t>
+  </si>
+  <si>
+    <t>Free delivery applies to all domestic orders with a value above PLN 150 gross. For orders below this amount, the courier shipping cost is PLN 14.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,81 +108,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,119 +412,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.1640625" customWidth="1"/>
+    <col min="2" max="2" width="53.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="170.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Nr pytania</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Pytanie</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Odpowiedź</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Jaki jest czas realizacji zamówienia w sklepie?</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Standardowy czas realizacji zamówienia wynosi od 1 do 3 dni roboczych. W przypadku przesyłek ekspresowych doręczenie następuje w ciągu 24 godzin od momentu nadania.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Jakie są warunki i procedury zwrotu towaru?</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Klient ma prawo odstąpić od umowy i zwrócić towar w ciągu 14 dni od momentu odebrania paczki bez podawania przyczyny. Towar musi być w stanie nienaruszonym wraz z oryginalnym opakowaniem i dowodem zakupu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Jak skontaktować się z działem pomocy technicznej i obsługi klienta?</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Dział obsługi klienta jest dostępny od poniedziałku do piątku w godzinach 8:00 - 18:00 pod numerem telefonu +48 22 123 45 67 oraz adresem e-mail: pomoc@twojafirma.pl.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Jakie formy płatności są akceptowane w sklepie?</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Obsługujemy szybkie płatności BLIK, karty płatnicze Visa i Mastercard, przelewy online PayU/Przelewy24 oraz płatność przy odbiorze (za pobraniem).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>W jaki sposób mogę zgłosić reklamację uszkodzonego produktu?</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Reklamację można zgłosić drogą elektroniczną, wysyłając formularz reklamacyjny ze zdjęciem wady na adres reklamacje@twojafirma.pl. Rozpatrzenie reklamacji trwa do 14 dni roboczych.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Czy oferujecie darmową dostawę i od jakiej kwoty?</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Darmowa dostawa przysługuje dla wszystkich zamówień krajowych o wartości powyżej 150 zł brutto. Dla zamówień poniżej tej kwoty koszt wysyłki kurierem wynosi 14 zł.</t>
-        </is>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>